<commit_message>
Add Robera Coffee Shop Survey to Week-01
</commit_message>
<xml_diff>
--- a/week-01/Ex4A_GTrends.xlsx
+++ b/week-01/Ex4A_GTrends.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yearuptemp-my.sharepoint.com/personal/hmerawi_my_yearupunited_org/Documents/Desktop/Documents/DataAnalytics/week-01/"/>
@@ -18,8 +18,11 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">GTrends_milkshake_hamburger_202!$A$1:$E$52</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -38,182 +41,182 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
+    <t>RegionID</t>
+  </si>
+  <si>
     <t>Region</t>
   </si>
   <si>
+    <t>Hamburger: (2/1/24 - 2/28/25)</t>
+  </si>
+  <si>
     <t>Milkshake: (2/1/24 - 2/28/25)</t>
   </si>
   <si>
-    <t>Hamburger: (2/1/24 - 2/28/25)</t>
-  </si>
-  <si>
     <t>Breakup: (2/1/24 - 2/28/25)</t>
   </si>
   <si>
+    <t># of regions</t>
+  </si>
+  <si>
+    <t>Alabama</t>
+  </si>
+  <si>
+    <t>Alaska</t>
+  </si>
+  <si>
+    <t>Arizona</t>
+  </si>
+  <si>
+    <t>Arkansas</t>
+  </si>
+  <si>
+    <t>California</t>
+  </si>
+  <si>
+    <t>Colorado</t>
+  </si>
+  <si>
+    <t>Connecticut</t>
+  </si>
+  <si>
+    <t>Delaware</t>
+  </si>
+  <si>
+    <t>District of Columbia</t>
+  </si>
+  <si>
+    <t>Florida</t>
+  </si>
+  <si>
+    <t>Georgia</t>
+  </si>
+  <si>
+    <t>Hawaii</t>
+  </si>
+  <si>
+    <t>Idaho</t>
+  </si>
+  <si>
+    <t>Illinois</t>
+  </si>
+  <si>
+    <t>Indiana</t>
+  </si>
+  <si>
+    <t>Iowa</t>
+  </si>
+  <si>
+    <t>Kansas</t>
+  </si>
+  <si>
+    <t>Kentucky</t>
+  </si>
+  <si>
+    <t>Louisiana</t>
+  </si>
+  <si>
+    <t>Maine</t>
+  </si>
+  <si>
+    <t>Maryland</t>
+  </si>
+  <si>
+    <t>Massachusetts</t>
+  </si>
+  <si>
+    <t>Michigan</t>
+  </si>
+  <si>
+    <t>Minnesota</t>
+  </si>
+  <si>
+    <t>Mississippi</t>
+  </si>
+  <si>
+    <t>Missouri</t>
+  </si>
+  <si>
+    <t>Montana</t>
+  </si>
+  <si>
+    <t>Nebraska</t>
+  </si>
+  <si>
+    <t>Nevada</t>
+  </si>
+  <si>
+    <t>New Hampshire</t>
+  </si>
+  <si>
+    <t>New Jersey</t>
+  </si>
+  <si>
+    <t>New Mexico</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>North Carolina</t>
+  </si>
+  <si>
+    <t>North Dakota</t>
+  </si>
+  <si>
+    <t>Ohio</t>
+  </si>
+  <si>
+    <t>Oklahoma</t>
+  </si>
+  <si>
+    <t>Oregon</t>
+  </si>
+  <si>
+    <t>Pennsylvania</t>
+  </si>
+  <si>
+    <t>Rhode Island</t>
+  </si>
+  <si>
     <t>South Carolina</t>
   </si>
   <si>
-    <t>Illinois</t>
-  </si>
-  <si>
-    <t>North Carolina</t>
+    <t>South Dakota</t>
   </si>
   <si>
     <t>Tennessee</t>
   </si>
   <si>
-    <t>Alabama</t>
-  </si>
-  <si>
-    <t>Kentucky</t>
-  </si>
-  <si>
-    <t>Indiana</t>
+    <t>Texas</t>
   </si>
   <si>
     <t>Utah</t>
   </si>
   <si>
-    <t>Georgia</t>
-  </si>
-  <si>
-    <t>Arkansas</t>
-  </si>
-  <si>
-    <t>Oklahoma</t>
-  </si>
-  <si>
-    <t>Delaware</t>
-  </si>
-  <si>
-    <t>Ohio</t>
+    <t>Vermont</t>
+  </si>
+  <si>
+    <t>Virginia</t>
+  </si>
+  <si>
+    <t>Washington</t>
   </si>
   <si>
     <t>West Virginia</t>
   </si>
   <si>
-    <t>Rhode Island</t>
-  </si>
-  <si>
-    <t>Pennsylvania</t>
-  </si>
-  <si>
-    <t>New Jersey</t>
-  </si>
-  <si>
-    <t>Connecticut</t>
-  </si>
-  <si>
-    <t>Nevada</t>
-  </si>
-  <si>
-    <t>Virginia</t>
-  </si>
-  <si>
-    <t>Maryland</t>
-  </si>
-  <si>
-    <t>Missouri</t>
-  </si>
-  <si>
-    <t>Florida</t>
-  </si>
-  <si>
-    <t>Michigan</t>
-  </si>
-  <si>
-    <t>Minnesota</t>
-  </si>
-  <si>
-    <t>Kansas</t>
-  </si>
-  <si>
-    <t>Arizona</t>
-  </si>
-  <si>
-    <t>Mississippi</t>
-  </si>
-  <si>
-    <t>Texas</t>
-  </si>
-  <si>
-    <t>Idaho</t>
-  </si>
-  <si>
-    <t>New Hampshire</t>
-  </si>
-  <si>
     <t>Wisconsin</t>
   </si>
   <si>
-    <t>Louisiana</t>
-  </si>
-  <si>
-    <t>Oregon</t>
-  </si>
-  <si>
-    <t>North Dakota</t>
-  </si>
-  <si>
-    <t>Nebraska</t>
-  </si>
-  <si>
-    <t>California</t>
-  </si>
-  <si>
-    <t>Iowa</t>
-  </si>
-  <si>
-    <t>New York</t>
-  </si>
-  <si>
-    <t>Colorado</t>
-  </si>
-  <si>
-    <t>Washington</t>
-  </si>
-  <si>
-    <t>Massachusetts</t>
-  </si>
-  <si>
-    <t>New Mexico</t>
-  </si>
-  <si>
-    <t>South Dakota</t>
-  </si>
-  <si>
     <t>Wyoming</t>
-  </si>
-  <si>
-    <t>Hawaii</t>
-  </si>
-  <si>
-    <t>Maine</t>
-  </si>
-  <si>
-    <t>Vermont</t>
-  </si>
-  <si>
-    <t>Montana</t>
-  </si>
-  <si>
-    <t>Alaska</t>
-  </si>
-  <si>
-    <t>District of Columbia</t>
-  </si>
-  <si>
-    <t># of regions</t>
-  </si>
-  <si>
-    <t>RegionID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1076,44 +1079,44 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8489D24C-89E2-46EF-98AF-AC6AA8C769DD}">
   <dimension ref="A1:H52"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="21.109375" customWidth="1"/>
-    <col min="3" max="4" width="27.6640625" customWidth="1"/>
-    <col min="5" max="5" width="25.21875" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="4" width="27.7109375" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="H1" s="2">
         <f>COUNTA(B2:B52)</f>
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1">
         <v>0.64</v>
@@ -1125,12 +1128,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="C3" s="1">
         <v>0.72</v>
@@ -1142,12 +1145,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1">
         <v>0.69</v>
@@ -1159,12 +1162,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C5" s="1">
         <v>0.64</v>
@@ -1176,12 +1179,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C6" s="1">
         <v>0.66</v>
@@ -1193,12 +1196,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C7" s="1">
         <v>0.67</v>
@@ -1210,12 +1213,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C8" s="1">
         <v>0.63</v>
@@ -1227,12 +1230,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1">
         <v>0.64</v>
@@ -1244,12 +1247,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="C10" s="1">
         <v>0.67</v>
@@ -1261,12 +1264,12 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C11" s="1">
         <v>0.63</v>
@@ -1278,12 +1281,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C12" s="1">
         <v>0.63</v>
@@ -1295,12 +1298,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C13" s="1">
         <v>0.72</v>
@@ -1312,12 +1315,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="C14" s="1">
         <v>0.67</v>
@@ -1329,12 +1332,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C15" s="1">
         <v>0.61</v>
@@ -1346,12 +1349,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C16" s="1">
         <v>0.64</v>
@@ -1363,12 +1366,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="C17" s="1">
         <v>0.68</v>
@@ -1380,12 +1383,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C18" s="1">
         <v>0.7</v>
@@ -1397,12 +1400,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C19" s="1">
         <v>0.64</v>
@@ -1414,12 +1417,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C20" s="1">
         <v>0.66</v>
@@ -1431,12 +1434,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C21" s="1">
         <v>0.7</v>
@@ -1448,12 +1451,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C22" s="1">
         <v>0.6</v>
@@ -1465,12 +1468,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="C23" s="1">
         <v>0.62</v>
@@ -1482,12 +1485,12 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C24" s="1">
         <v>0.69</v>
@@ -1499,12 +1502,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C25" s="1">
         <v>0.66</v>
@@ -1516,12 +1519,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C26" s="1">
         <v>0.68</v>
@@ -1533,12 +1536,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C27" s="1">
         <v>0.67</v>
@@ -1550,12 +1553,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C28" s="1">
         <v>0.75</v>
@@ -1567,12 +1570,12 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C29" s="1">
         <v>0.69</v>
@@ -1584,12 +1587,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C30" s="1">
         <v>0.68</v>
@@ -1601,12 +1604,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C31" s="1">
         <v>0.64</v>
@@ -1618,12 +1621,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C32" s="1">
         <v>0.6</v>
@@ -1635,12 +1638,12 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C33" s="1">
         <v>0.68</v>
@@ -1652,12 +1655,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C34" s="1">
         <v>0.64</v>
@@ -1669,12 +1672,12 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C35" s="1">
         <v>0.63</v>
@@ -1686,12 +1689,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C36" s="1">
         <v>0.69</v>
@@ -1703,12 +1706,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="C37" s="1">
         <v>0.64</v>
@@ -1720,12 +1723,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="C38" s="1">
         <v>0.69</v>
@@ -1737,12 +1740,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C39" s="1">
         <v>0.68</v>
@@ -1754,12 +1757,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="C40" s="1">
         <v>0.61</v>
@@ -1771,12 +1774,12 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="C41" s="1">
         <v>0.64</v>
@@ -1788,12 +1791,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="C42" s="1">
         <v>0.66</v>
@@ -1805,7 +1808,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1822,12 +1825,12 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="C44" s="1">
         <v>0.65</v>
@@ -1839,12 +1842,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="C45" s="1">
         <v>0.67</v>
@@ -1856,12 +1859,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="C46" s="1">
         <v>0.67</v>
@@ -1873,7 +1876,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1890,12 +1893,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C48" s="1">
         <v>0.65</v>
@@ -1907,12 +1910,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C49" s="1">
         <v>0.68</v>
@@ -1924,12 +1927,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="C50" s="1">
         <v>0.64</v>
@@ -1941,12 +1944,12 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="C51" s="1">
         <v>0.66</v>
@@ -1958,12 +1961,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C52" s="1">
         <v>0.71</v>

</xml_diff>